<commit_message>
Add Top Priority card to Admin-Queue dashboard
Adds a dynamic 'Top Priority' KPI card that surfaces the most urgent
priority currently set in the Priority column via an IFS formula, with
conditional formatting that colors the value to match the priority.
</commit_message>
<xml_diff>
--- a/Admin-Queue.xlsx
+++ b/Admin-Queue.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Admin Queue" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Admin Queue'!$A$10:$I$71</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Admin Queue'!$A$15:$I$76</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="13">
+  <fonts count="14">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -73,6 +73,11 @@
     <font>
       <b val="1"/>
       <color rgb="001F2A44"/>
+      <sz val="22"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F2A44"/>
       <sz val="10"/>
     </font>
     <font>
@@ -84,7 +89,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -123,11 +128,16 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="001F2A44"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00F2F5FA"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="11">
+  <borders count="14">
     <border>
       <left/>
       <right/>
@@ -226,6 +236,28 @@
       </bottom>
     </border>
     <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D8DEE9"/>
+      </top>
+      <bottom/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00D8DEE9"/>
+      </bottom>
+    </border>
+    <border>
       <left style="thin">
         <color rgb="00D8DEE9"/>
       </left>
@@ -243,7 +275,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -282,24 +314,79 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="8" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="12">
+  <dxfs count="16">
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="00D64545"/>
+        <sz val="22"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFFFFF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="00E0892B"/>
+        <sz val="22"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFFFFF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="009A7B0A"/>
+        <sz val="22"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFFFFF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="003FA34D"/>
+        <sz val="22"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFFFFF"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -778,7 +865,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I71"/>
+  <dimension ref="A1:I76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -905,980 +992,1012 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="22" customHeight="1">
-      <c r="A10" s="20" t="inlineStr">
+    <row r="9" ht="5" customHeight="1">
+      <c r="A9" s="20" t="n"/>
+      <c r="B9" s="21" t="n"/>
+      <c r="C9" s="4" t="n"/>
+    </row>
+    <row r="10" ht="34" customHeight="1">
+      <c r="A10" s="22">
+        <f>IFS(COUNTIF(D:D,"Critical")&gt;0,"Critical",COUNTIF(D:D,"High")&gt;0,"High",COUNTIF(D:D,"Medium")&gt;0,"Medium",COUNTIF(D:D,"Low")&gt;0,"Low",TRUE,"No priority set")</f>
+        <v/>
+      </c>
+      <c r="B10" s="23" t="n"/>
+      <c r="C10" s="10" t="n"/>
+    </row>
+    <row r="11" ht="15" customHeight="1">
+      <c r="A11" s="15" t="inlineStr">
+        <is>
+          <t>TOP PRIORITY</t>
+        </is>
+      </c>
+      <c r="B11" s="23" t="n"/>
+      <c r="C11" s="10" t="n"/>
+    </row>
+    <row r="12" ht="14" customHeight="1">
+      <c r="A12" s="17" t="inlineStr">
+        <is>
+          <t>Highest in the queue right now</t>
+        </is>
+      </c>
+      <c r="B12" s="24" t="n"/>
+      <c r="C12" s="18" t="n"/>
+    </row>
+    <row r="15" ht="22" customHeight="1">
+      <c r="A15" s="25" t="inlineStr">
         <is>
           <t>Request</t>
         </is>
       </c>
-      <c r="B10" s="20" t="inlineStr">
+      <c r="B15" s="25" t="inlineStr">
         <is>
           <t>Requester</t>
         </is>
       </c>
-      <c r="C10" s="20" t="inlineStr">
+      <c r="C15" s="25" t="inlineStr">
         <is>
           <t>Application(s)</t>
         </is>
       </c>
-      <c r="D10" s="20" t="inlineStr">
+      <c r="D15" s="25" t="inlineStr">
         <is>
           <t>Priority</t>
         </is>
       </c>
-      <c r="E10" s="20" t="inlineStr">
+      <c r="E15" s="25" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F10" s="20" t="inlineStr">
+      <c r="F15" s="25" t="inlineStr">
         <is>
           <t>Jira #</t>
         </is>
       </c>
-      <c r="G10" s="20" t="inlineStr">
+      <c r="G15" s="25" t="inlineStr">
         <is>
           <t>Sprint</t>
         </is>
       </c>
-      <c r="H10" s="20" t="inlineStr">
+      <c r="H15" s="25" t="inlineStr">
         <is>
           <t>Submitted</t>
         </is>
       </c>
-      <c r="I10" s="20" t="inlineStr">
+      <c r="I15" s="25" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="22" customHeight="1">
-      <c r="A11" s="21" t="inlineStr">
+    <row r="16" ht="22" customHeight="1">
+      <c r="A16" s="26" t="inlineStr">
         <is>
           <t>Agent — Screen Pop Customization</t>
         </is>
       </c>
-      <c r="B11" s="22" t="inlineStr">
+      <c r="B16" s="27" t="inlineStr">
         <is>
           <t>Sarah M.</t>
         </is>
       </c>
-      <c r="C11" s="22" t="inlineStr">
+      <c r="C16" s="27" t="inlineStr">
         <is>
           <t>Agent</t>
         </is>
       </c>
-      <c r="D11" s="23" t="inlineStr">
+      <c r="D16" s="28" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E11" s="23" t="inlineStr">
+      <c r="E16" s="28" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
       </c>
-      <c r="F11" s="22" t="inlineStr">
+      <c r="F16" s="27" t="inlineStr">
         <is>
           <t>DEMO-482</t>
         </is>
       </c>
-      <c r="G11" s="22" t="inlineStr">
+      <c r="G16" s="27" t="inlineStr">
         <is>
           <t>Sprint 44</t>
         </is>
       </c>
-      <c r="H11" s="22" t="inlineStr">
+      <c r="H16" s="27" t="inlineStr">
         <is>
           <t>May 2</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="21" t="inlineStr">
+    <row r="17" ht="22" customHeight="1">
+      <c r="A17" s="26" t="inlineStr">
         <is>
           <t>WFM — Real-Time Adherence Dashboard</t>
         </is>
       </c>
-      <c r="B12" s="22" t="inlineStr">
+      <c r="B17" s="27" t="inlineStr">
         <is>
           <t>James T.</t>
         </is>
       </c>
-      <c r="C12" s="22" t="inlineStr">
+      <c r="C17" s="27" t="inlineStr">
         <is>
           <t>WFM, Supervisor</t>
         </is>
       </c>
-      <c r="D12" s="23" t="inlineStr">
+      <c r="D17" s="28" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
       </c>
-      <c r="E12" s="23" t="inlineStr">
+      <c r="E17" s="28" t="inlineStr">
         <is>
           <t>In Progress</t>
         </is>
       </c>
-      <c r="F12" s="22" t="inlineStr">
+      <c r="F17" s="27" t="inlineStr">
         <is>
           <t>DEMO-479</t>
         </is>
       </c>
-      <c r="G12" s="22" t="inlineStr">
+      <c r="G17" s="27" t="inlineStr">
         <is>
           <t>Sprint 44</t>
         </is>
       </c>
-      <c r="H12" s="22" t="inlineStr">
+      <c r="H17" s="27" t="inlineStr">
         <is>
           <t>Apr 30</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="22" customHeight="1">
-      <c r="A13" s="21" t="inlineStr">
+    <row r="18" ht="22" customHeight="1">
+      <c r="A18" s="26" t="inlineStr">
         <is>
           <t>QM — AI Evaluation Scorecard</t>
         </is>
       </c>
-      <c r="B13" s="22" t="inlineStr">
+      <c r="B18" s="27" t="inlineStr">
         <is>
           <t>Priya K.</t>
         </is>
       </c>
-      <c r="C13" s="22" t="inlineStr">
+      <c r="C18" s="27" t="inlineStr">
         <is>
           <t>Quality Management</t>
         </is>
       </c>
-      <c r="D13" s="23" t="inlineStr">
+      <c r="D18" s="28" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E13" s="23" t="inlineStr">
+      <c r="E18" s="28" t="inlineStr">
         <is>
           <t>Approved</t>
         </is>
       </c>
-      <c r="F13" s="22" t="inlineStr">
+      <c r="F18" s="27" t="inlineStr">
         <is>
           <t>DEMO-491</t>
         </is>
       </c>
-      <c r="G13" s="22" t="inlineStr">
+      <c r="G18" s="27" t="inlineStr">
         <is>
           <t>Sprint 45</t>
         </is>
       </c>
-      <c r="H13" s="22" t="inlineStr">
+      <c r="H18" s="27" t="inlineStr">
         <is>
           <t>May 4</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="22" customHeight="1">
-      <c r="A14" s="21" t="inlineStr">
+    <row r="19" ht="22" customHeight="1">
+      <c r="A19" s="26" t="inlineStr">
         <is>
           <t>Supervisor — Live Monitoring Panel</t>
         </is>
       </c>
-      <c r="B14" s="22" t="inlineStr">
+      <c r="B19" s="27" t="inlineStr">
         <is>
           <t>Marcus L.</t>
         </is>
       </c>
-      <c r="C14" s="22" t="inlineStr">
+      <c r="C19" s="27" t="inlineStr">
         <is>
           <t>Supervisor</t>
         </is>
       </c>
-      <c r="D14" s="23" t="inlineStr">
+      <c r="D19" s="28" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E14" s="23" t="inlineStr">
+      <c r="E19" s="28" t="inlineStr">
         <is>
           <t>In Review</t>
         </is>
       </c>
-      <c r="F14" s="22" t="inlineStr">
+      <c r="F19" s="27" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G14" s="22" t="inlineStr">
+      <c r="G19" s="27" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H14" s="22" t="inlineStr">
+      <c r="H19" s="27" t="inlineStr">
         <is>
           <t>May 5</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="22" customHeight="1">
-      <c r="A15" s="21" t="inlineStr">
+    <row r="20" ht="22" customHeight="1">
+      <c r="A20" s="26" t="inlineStr">
         <is>
           <t>Interactions Hub — Recording Playback</t>
         </is>
       </c>
-      <c r="B15" s="22" t="inlineStr">
+      <c r="B20" s="27" t="inlineStr">
         <is>
           <t>Dana W.</t>
         </is>
       </c>
-      <c r="C15" s="22" t="inlineStr">
+      <c r="C20" s="27" t="inlineStr">
         <is>
           <t>Interactions Hub</t>
         </is>
       </c>
-      <c r="D15" s="23" t="inlineStr">
+      <c r="D20" s="28" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="E15" s="23" t="inlineStr">
+      <c r="E20" s="28" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="F15" s="22" t="inlineStr">
+      <c r="F20" s="27" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G15" s="22" t="inlineStr">
+      <c r="G20" s="27" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H15" s="22" t="inlineStr">
+      <c r="H20" s="27" t="inlineStr">
         <is>
           <t>May 6</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="22" customHeight="1">
-      <c r="A16" s="21" t="inlineStr">
+    <row r="21" ht="22" customHeight="1">
+      <c r="A21" s="26" t="inlineStr">
         <is>
           <t>Smart Reach — Campaign Builder Flow</t>
         </is>
       </c>
-      <c r="B16" s="22" t="inlineStr">
+      <c r="B21" s="27" t="inlineStr">
         <is>
           <t>Jordan B.</t>
         </is>
       </c>
-      <c r="C16" s="22" t="inlineStr">
+      <c r="C21" s="27" t="inlineStr">
         <is>
           <t>Smart Reach</t>
         </is>
       </c>
-      <c r="D16" s="23" t="inlineStr">
+      <c r="D21" s="28" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E16" s="23" t="inlineStr">
+      <c r="E21" s="28" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="F16" s="22" t="inlineStr">
+      <c r="F21" s="27" t="inlineStr">
         <is>
           <t>DEMO-465</t>
         </is>
       </c>
-      <c r="G16" s="22" t="inlineStr">
+      <c r="G21" s="27" t="inlineStr">
         <is>
           <t>Sprint 43</t>
         </is>
       </c>
-      <c r="H16" s="22" t="inlineStr">
+      <c r="H21" s="27" t="inlineStr">
         <is>
           <t>Apr 22</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="22" customHeight="1">
-      <c r="A17" s="21" t="inlineStr">
+    <row r="22" ht="22" customHeight="1">
+      <c r="A22" s="26" t="inlineStr">
         <is>
           <t>My Zone — Schedule Visibility</t>
         </is>
       </c>
-      <c r="B17" s="22" t="inlineStr">
+      <c r="B22" s="27" t="inlineStr">
         <is>
           <t>Sarah M.</t>
         </is>
       </c>
-      <c r="C17" s="22" t="inlineStr">
+      <c r="C22" s="27" t="inlineStr">
         <is>
           <t>My Zone</t>
         </is>
       </c>
-      <c r="D17" s="23" t="inlineStr">
+      <c r="D22" s="28" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E17" s="23" t="inlineStr">
+      <c r="E22" s="28" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="F17" s="22" t="inlineStr">
+      <c r="F22" s="27" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G17" s="22" t="inlineStr">
+      <c r="G22" s="27" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H17" s="22" t="inlineStr">
+      <c r="H22" s="27" t="inlineStr">
         <is>
           <t>May 6</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="22" customHeight="1">
-      <c r="A18" s="21" t="inlineStr">
+    <row r="23" ht="22" customHeight="1">
+      <c r="A23" s="26" t="inlineStr">
         <is>
           <t>Agent — After Call Work Timer</t>
         </is>
       </c>
-      <c r="B18" s="22" t="inlineStr">
+      <c r="B23" s="27" t="inlineStr">
         <is>
           <t>Priya K.</t>
         </is>
       </c>
-      <c r="C18" s="22" t="inlineStr">
+      <c r="C23" s="27" t="inlineStr">
         <is>
           <t>Agent</t>
         </is>
       </c>
-      <c r="D18" s="23" t="inlineStr">
+      <c r="D23" s="28" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E18" s="23" t="inlineStr">
+      <c r="E23" s="28" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="F18" s="22" t="inlineStr">
+      <c r="F23" s="27" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G18" s="22" t="inlineStr">
+      <c r="G23" s="27" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H18" s="22" t="inlineStr">
+      <c r="H23" s="27" t="inlineStr">
         <is>
           <t>May 6</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="20" customHeight="1">
-      <c r="A19" s="24" t="n"/>
-      <c r="B19" s="24" t="n"/>
-      <c r="C19" s="24" t="n"/>
-      <c r="D19" s="24" t="n"/>
-      <c r="E19" s="24" t="n"/>
-      <c r="F19" s="24" t="n"/>
-      <c r="G19" s="24" t="n"/>
-      <c r="H19" s="24" t="n"/>
-      <c r="I19" s="24" t="n"/>
-    </row>
-    <row r="20" ht="20" customHeight="1">
-      <c r="A20" s="24" t="n"/>
-      <c r="B20" s="24" t="n"/>
-      <c r="C20" s="24" t="n"/>
-      <c r="D20" s="24" t="n"/>
-      <c r="E20" s="24" t="n"/>
-      <c r="F20" s="24" t="n"/>
-      <c r="G20" s="24" t="n"/>
-      <c r="H20" s="24" t="n"/>
-      <c r="I20" s="24" t="n"/>
-    </row>
-    <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="24" t="n"/>
-      <c r="B21" s="24" t="n"/>
-      <c r="C21" s="24" t="n"/>
-      <c r="D21" s="24" t="n"/>
-      <c r="E21" s="24" t="n"/>
-      <c r="F21" s="24" t="n"/>
-      <c r="G21" s="24" t="n"/>
-      <c r="H21" s="24" t="n"/>
-      <c r="I21" s="24" t="n"/>
-    </row>
-    <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="24" t="n"/>
-      <c r="B22" s="24" t="n"/>
-      <c r="C22" s="24" t="n"/>
-      <c r="D22" s="24" t="n"/>
-      <c r="E22" s="24" t="n"/>
-      <c r="F22" s="24" t="n"/>
-      <c r="G22" s="24" t="n"/>
-      <c r="H22" s="24" t="n"/>
-      <c r="I22" s="24" t="n"/>
-    </row>
-    <row r="23" ht="20" customHeight="1">
-      <c r="A23" s="24" t="n"/>
-      <c r="B23" s="24" t="n"/>
-      <c r="C23" s="24" t="n"/>
-      <c r="D23" s="24" t="n"/>
-      <c r="E23" s="24" t="n"/>
-      <c r="F23" s="24" t="n"/>
-      <c r="G23" s="24" t="n"/>
-      <c r="H23" s="24" t="n"/>
-      <c r="I23" s="24" t="n"/>
-    </row>
     <row r="24" ht="20" customHeight="1">
-      <c r="A24" s="24" t="n"/>
-      <c r="B24" s="24" t="n"/>
-      <c r="C24" s="24" t="n"/>
-      <c r="D24" s="24" t="n"/>
-      <c r="E24" s="24" t="n"/>
-      <c r="F24" s="24" t="n"/>
-      <c r="G24" s="24" t="n"/>
-      <c r="H24" s="24" t="n"/>
-      <c r="I24" s="24" t="n"/>
+      <c r="A24" s="29" t="n"/>
+      <c r="B24" s="29" t="n"/>
+      <c r="C24" s="29" t="n"/>
+      <c r="D24" s="29" t="n"/>
+      <c r="E24" s="29" t="n"/>
+      <c r="F24" s="29" t="n"/>
+      <c r="G24" s="29" t="n"/>
+      <c r="H24" s="29" t="n"/>
+      <c r="I24" s="29" t="n"/>
     </row>
     <row r="25" ht="20" customHeight="1">
-      <c r="A25" s="24" t="n"/>
-      <c r="B25" s="24" t="n"/>
-      <c r="C25" s="24" t="n"/>
-      <c r="D25" s="24" t="n"/>
-      <c r="E25" s="24" t="n"/>
-      <c r="F25" s="24" t="n"/>
-      <c r="G25" s="24" t="n"/>
-      <c r="H25" s="24" t="n"/>
-      <c r="I25" s="24" t="n"/>
+      <c r="A25" s="29" t="n"/>
+      <c r="B25" s="29" t="n"/>
+      <c r="C25" s="29" t="n"/>
+      <c r="D25" s="29" t="n"/>
+      <c r="E25" s="29" t="n"/>
+      <c r="F25" s="29" t="n"/>
+      <c r="G25" s="29" t="n"/>
+      <c r="H25" s="29" t="n"/>
+      <c r="I25" s="29" t="n"/>
     </row>
     <row r="26" ht="20" customHeight="1">
-      <c r="A26" s="24" t="n"/>
-      <c r="B26" s="24" t="n"/>
-      <c r="C26" s="24" t="n"/>
-      <c r="D26" s="24" t="n"/>
-      <c r="E26" s="24" t="n"/>
-      <c r="F26" s="24" t="n"/>
-      <c r="G26" s="24" t="n"/>
-      <c r="H26" s="24" t="n"/>
-      <c r="I26" s="24" t="n"/>
+      <c r="A26" s="29" t="n"/>
+      <c r="B26" s="29" t="n"/>
+      <c r="C26" s="29" t="n"/>
+      <c r="D26" s="29" t="n"/>
+      <c r="E26" s="29" t="n"/>
+      <c r="F26" s="29" t="n"/>
+      <c r="G26" s="29" t="n"/>
+      <c r="H26" s="29" t="n"/>
+      <c r="I26" s="29" t="n"/>
     </row>
     <row r="27" ht="20" customHeight="1">
-      <c r="A27" s="24" t="n"/>
-      <c r="B27" s="24" t="n"/>
-      <c r="C27" s="24" t="n"/>
-      <c r="D27" s="24" t="n"/>
-      <c r="E27" s="24" t="n"/>
-      <c r="F27" s="24" t="n"/>
-      <c r="G27" s="24" t="n"/>
-      <c r="H27" s="24" t="n"/>
-      <c r="I27" s="24" t="n"/>
+      <c r="A27" s="29" t="n"/>
+      <c r="B27" s="29" t="n"/>
+      <c r="C27" s="29" t="n"/>
+      <c r="D27" s="29" t="n"/>
+      <c r="E27" s="29" t="n"/>
+      <c r="F27" s="29" t="n"/>
+      <c r="G27" s="29" t="n"/>
+      <c r="H27" s="29" t="n"/>
+      <c r="I27" s="29" t="n"/>
     </row>
     <row r="28" ht="20" customHeight="1">
-      <c r="A28" s="24" t="n"/>
-      <c r="B28" s="24" t="n"/>
-      <c r="C28" s="24" t="n"/>
-      <c r="D28" s="24" t="n"/>
-      <c r="E28" s="24" t="n"/>
-      <c r="F28" s="24" t="n"/>
-      <c r="G28" s="24" t="n"/>
-      <c r="H28" s="24" t="n"/>
-      <c r="I28" s="24" t="n"/>
+      <c r="A28" s="29" t="n"/>
+      <c r="B28" s="29" t="n"/>
+      <c r="C28" s="29" t="n"/>
+      <c r="D28" s="29" t="n"/>
+      <c r="E28" s="29" t="n"/>
+      <c r="F28" s="29" t="n"/>
+      <c r="G28" s="29" t="n"/>
+      <c r="H28" s="29" t="n"/>
+      <c r="I28" s="29" t="n"/>
     </row>
     <row r="29" ht="20" customHeight="1">
-      <c r="A29" s="24" t="n"/>
-      <c r="B29" s="24" t="n"/>
-      <c r="C29" s="24" t="n"/>
-      <c r="D29" s="24" t="n"/>
-      <c r="E29" s="24" t="n"/>
-      <c r="F29" s="24" t="n"/>
-      <c r="G29" s="24" t="n"/>
-      <c r="H29" s="24" t="n"/>
-      <c r="I29" s="24" t="n"/>
+      <c r="A29" s="29" t="n"/>
+      <c r="B29" s="29" t="n"/>
+      <c r="C29" s="29" t="n"/>
+      <c r="D29" s="29" t="n"/>
+      <c r="E29" s="29" t="n"/>
+      <c r="F29" s="29" t="n"/>
+      <c r="G29" s="29" t="n"/>
+      <c r="H29" s="29" t="n"/>
+      <c r="I29" s="29" t="n"/>
     </row>
     <row r="30" ht="20" customHeight="1">
-      <c r="A30" s="24" t="n"/>
-      <c r="B30" s="24" t="n"/>
-      <c r="C30" s="24" t="n"/>
-      <c r="D30" s="24" t="n"/>
-      <c r="E30" s="24" t="n"/>
-      <c r="F30" s="24" t="n"/>
-      <c r="G30" s="24" t="n"/>
-      <c r="H30" s="24" t="n"/>
-      <c r="I30" s="24" t="n"/>
+      <c r="A30" s="29" t="n"/>
+      <c r="B30" s="29" t="n"/>
+      <c r="C30" s="29" t="n"/>
+      <c r="D30" s="29" t="n"/>
+      <c r="E30" s="29" t="n"/>
+      <c r="F30" s="29" t="n"/>
+      <c r="G30" s="29" t="n"/>
+      <c r="H30" s="29" t="n"/>
+      <c r="I30" s="29" t="n"/>
     </row>
     <row r="31" ht="20" customHeight="1">
-      <c r="A31" s="24" t="n"/>
-      <c r="B31" s="24" t="n"/>
-      <c r="C31" s="24" t="n"/>
-      <c r="D31" s="24" t="n"/>
-      <c r="E31" s="24" t="n"/>
-      <c r="F31" s="24" t="n"/>
-      <c r="G31" s="24" t="n"/>
-      <c r="H31" s="24" t="n"/>
-      <c r="I31" s="24" t="n"/>
+      <c r="A31" s="29" t="n"/>
+      <c r="B31" s="29" t="n"/>
+      <c r="C31" s="29" t="n"/>
+      <c r="D31" s="29" t="n"/>
+      <c r="E31" s="29" t="n"/>
+      <c r="F31" s="29" t="n"/>
+      <c r="G31" s="29" t="n"/>
+      <c r="H31" s="29" t="n"/>
+      <c r="I31" s="29" t="n"/>
     </row>
     <row r="32" ht="20" customHeight="1">
-      <c r="A32" s="24" t="n"/>
-      <c r="B32" s="24" t="n"/>
-      <c r="C32" s="24" t="n"/>
-      <c r="D32" s="24" t="n"/>
-      <c r="E32" s="24" t="n"/>
-      <c r="F32" s="24" t="n"/>
-      <c r="G32" s="24" t="n"/>
-      <c r="H32" s="24" t="n"/>
-      <c r="I32" s="24" t="n"/>
+      <c r="A32" s="29" t="n"/>
+      <c r="B32" s="29" t="n"/>
+      <c r="C32" s="29" t="n"/>
+      <c r="D32" s="29" t="n"/>
+      <c r="E32" s="29" t="n"/>
+      <c r="F32" s="29" t="n"/>
+      <c r="G32" s="29" t="n"/>
+      <c r="H32" s="29" t="n"/>
+      <c r="I32" s="29" t="n"/>
     </row>
     <row r="33" ht="20" customHeight="1">
-      <c r="A33" s="24" t="n"/>
-      <c r="B33" s="24" t="n"/>
-      <c r="C33" s="24" t="n"/>
-      <c r="D33" s="24" t="n"/>
-      <c r="E33" s="24" t="n"/>
-      <c r="F33" s="24" t="n"/>
-      <c r="G33" s="24" t="n"/>
-      <c r="H33" s="24" t="n"/>
-      <c r="I33" s="24" t="n"/>
+      <c r="A33" s="29" t="n"/>
+      <c r="B33" s="29" t="n"/>
+      <c r="C33" s="29" t="n"/>
+      <c r="D33" s="29" t="n"/>
+      <c r="E33" s="29" t="n"/>
+      <c r="F33" s="29" t="n"/>
+      <c r="G33" s="29" t="n"/>
+      <c r="H33" s="29" t="n"/>
+      <c r="I33" s="29" t="n"/>
     </row>
     <row r="34" ht="20" customHeight="1">
-      <c r="A34" s="24" t="n"/>
-      <c r="B34" s="24" t="n"/>
-      <c r="C34" s="24" t="n"/>
-      <c r="D34" s="24" t="n"/>
-      <c r="E34" s="24" t="n"/>
-      <c r="F34" s="24" t="n"/>
-      <c r="G34" s="24" t="n"/>
-      <c r="H34" s="24" t="n"/>
-      <c r="I34" s="24" t="n"/>
+      <c r="A34" s="29" t="n"/>
+      <c r="B34" s="29" t="n"/>
+      <c r="C34" s="29" t="n"/>
+      <c r="D34" s="29" t="n"/>
+      <c r="E34" s="29" t="n"/>
+      <c r="F34" s="29" t="n"/>
+      <c r="G34" s="29" t="n"/>
+      <c r="H34" s="29" t="n"/>
+      <c r="I34" s="29" t="n"/>
     </row>
     <row r="35" ht="20" customHeight="1">
-      <c r="A35" s="24" t="n"/>
-      <c r="B35" s="24" t="n"/>
-      <c r="C35" s="24" t="n"/>
-      <c r="D35" s="24" t="n"/>
-      <c r="E35" s="24" t="n"/>
-      <c r="F35" s="24" t="n"/>
-      <c r="G35" s="24" t="n"/>
-      <c r="H35" s="24" t="n"/>
-      <c r="I35" s="24" t="n"/>
+      <c r="A35" s="29" t="n"/>
+      <c r="B35" s="29" t="n"/>
+      <c r="C35" s="29" t="n"/>
+      <c r="D35" s="29" t="n"/>
+      <c r="E35" s="29" t="n"/>
+      <c r="F35" s="29" t="n"/>
+      <c r="G35" s="29" t="n"/>
+      <c r="H35" s="29" t="n"/>
+      <c r="I35" s="29" t="n"/>
     </row>
     <row r="36" ht="20" customHeight="1">
-      <c r="A36" s="24" t="n"/>
-      <c r="B36" s="24" t="n"/>
-      <c r="C36" s="24" t="n"/>
-      <c r="D36" s="24" t="n"/>
-      <c r="E36" s="24" t="n"/>
-      <c r="F36" s="24" t="n"/>
-      <c r="G36" s="24" t="n"/>
-      <c r="H36" s="24" t="n"/>
-      <c r="I36" s="24" t="n"/>
+      <c r="A36" s="29" t="n"/>
+      <c r="B36" s="29" t="n"/>
+      <c r="C36" s="29" t="n"/>
+      <c r="D36" s="29" t="n"/>
+      <c r="E36" s="29" t="n"/>
+      <c r="F36" s="29" t="n"/>
+      <c r="G36" s="29" t="n"/>
+      <c r="H36" s="29" t="n"/>
+      <c r="I36" s="29" t="n"/>
     </row>
     <row r="37" ht="20" customHeight="1">
-      <c r="A37" s="24" t="n"/>
-      <c r="B37" s="24" t="n"/>
-      <c r="C37" s="24" t="n"/>
-      <c r="D37" s="24" t="n"/>
-      <c r="E37" s="24" t="n"/>
-      <c r="F37" s="24" t="n"/>
-      <c r="G37" s="24" t="n"/>
-      <c r="H37" s="24" t="n"/>
-      <c r="I37" s="24" t="n"/>
+      <c r="A37" s="29" t="n"/>
+      <c r="B37" s="29" t="n"/>
+      <c r="C37" s="29" t="n"/>
+      <c r="D37" s="29" t="n"/>
+      <c r="E37" s="29" t="n"/>
+      <c r="F37" s="29" t="n"/>
+      <c r="G37" s="29" t="n"/>
+      <c r="H37" s="29" t="n"/>
+      <c r="I37" s="29" t="n"/>
     </row>
     <row r="38" ht="20" customHeight="1">
-      <c r="A38" s="24" t="n"/>
-      <c r="B38" s="24" t="n"/>
-      <c r="C38" s="24" t="n"/>
-      <c r="D38" s="24" t="n"/>
-      <c r="E38" s="24" t="n"/>
-      <c r="F38" s="24" t="n"/>
-      <c r="G38" s="24" t="n"/>
-      <c r="H38" s="24" t="n"/>
-      <c r="I38" s="24" t="n"/>
+      <c r="A38" s="29" t="n"/>
+      <c r="B38" s="29" t="n"/>
+      <c r="C38" s="29" t="n"/>
+      <c r="D38" s="29" t="n"/>
+      <c r="E38" s="29" t="n"/>
+      <c r="F38" s="29" t="n"/>
+      <c r="G38" s="29" t="n"/>
+      <c r="H38" s="29" t="n"/>
+      <c r="I38" s="29" t="n"/>
     </row>
     <row r="39" ht="20" customHeight="1">
-      <c r="A39" s="24" t="n"/>
-      <c r="B39" s="24" t="n"/>
-      <c r="C39" s="24" t="n"/>
-      <c r="D39" s="24" t="n"/>
-      <c r="E39" s="24" t="n"/>
-      <c r="F39" s="24" t="n"/>
-      <c r="G39" s="24" t="n"/>
-      <c r="H39" s="24" t="n"/>
-      <c r="I39" s="24" t="n"/>
+      <c r="A39" s="29" t="n"/>
+      <c r="B39" s="29" t="n"/>
+      <c r="C39" s="29" t="n"/>
+      <c r="D39" s="29" t="n"/>
+      <c r="E39" s="29" t="n"/>
+      <c r="F39" s="29" t="n"/>
+      <c r="G39" s="29" t="n"/>
+      <c r="H39" s="29" t="n"/>
+      <c r="I39" s="29" t="n"/>
     </row>
     <row r="40" ht="20" customHeight="1">
-      <c r="A40" s="24" t="n"/>
-      <c r="B40" s="24" t="n"/>
-      <c r="C40" s="24" t="n"/>
-      <c r="D40" s="24" t="n"/>
-      <c r="E40" s="24" t="n"/>
-      <c r="F40" s="24" t="n"/>
-      <c r="G40" s="24" t="n"/>
-      <c r="H40" s="24" t="n"/>
-      <c r="I40" s="24" t="n"/>
+      <c r="A40" s="29" t="n"/>
+      <c r="B40" s="29" t="n"/>
+      <c r="C40" s="29" t="n"/>
+      <c r="D40" s="29" t="n"/>
+      <c r="E40" s="29" t="n"/>
+      <c r="F40" s="29" t="n"/>
+      <c r="G40" s="29" t="n"/>
+      <c r="H40" s="29" t="n"/>
+      <c r="I40" s="29" t="n"/>
     </row>
     <row r="41" ht="20" customHeight="1">
-      <c r="A41" s="24" t="n"/>
-      <c r="B41" s="24" t="n"/>
-      <c r="C41" s="24" t="n"/>
-      <c r="D41" s="24" t="n"/>
-      <c r="E41" s="24" t="n"/>
-      <c r="F41" s="24" t="n"/>
-      <c r="G41" s="24" t="n"/>
-      <c r="H41" s="24" t="n"/>
-      <c r="I41" s="24" t="n"/>
+      <c r="A41" s="29" t="n"/>
+      <c r="B41" s="29" t="n"/>
+      <c r="C41" s="29" t="n"/>
+      <c r="D41" s="29" t="n"/>
+      <c r="E41" s="29" t="n"/>
+      <c r="F41" s="29" t="n"/>
+      <c r="G41" s="29" t="n"/>
+      <c r="H41" s="29" t="n"/>
+      <c r="I41" s="29" t="n"/>
     </row>
     <row r="42" ht="20" customHeight="1">
-      <c r="A42" s="24" t="n"/>
-      <c r="B42" s="24" t="n"/>
-      <c r="C42" s="24" t="n"/>
-      <c r="D42" s="24" t="n"/>
-      <c r="E42" s="24" t="n"/>
-      <c r="F42" s="24" t="n"/>
-      <c r="G42" s="24" t="n"/>
-      <c r="H42" s="24" t="n"/>
-      <c r="I42" s="24" t="n"/>
+      <c r="A42" s="29" t="n"/>
+      <c r="B42" s="29" t="n"/>
+      <c r="C42" s="29" t="n"/>
+      <c r="D42" s="29" t="n"/>
+      <c r="E42" s="29" t="n"/>
+      <c r="F42" s="29" t="n"/>
+      <c r="G42" s="29" t="n"/>
+      <c r="H42" s="29" t="n"/>
+      <c r="I42" s="29" t="n"/>
     </row>
     <row r="43" ht="20" customHeight="1">
-      <c r="A43" s="24" t="n"/>
-      <c r="B43" s="24" t="n"/>
-      <c r="C43" s="24" t="n"/>
-      <c r="D43" s="24" t="n"/>
-      <c r="E43" s="24" t="n"/>
-      <c r="F43" s="24" t="n"/>
-      <c r="G43" s="24" t="n"/>
-      <c r="H43" s="24" t="n"/>
-      <c r="I43" s="24" t="n"/>
+      <c r="A43" s="29" t="n"/>
+      <c r="B43" s="29" t="n"/>
+      <c r="C43" s="29" t="n"/>
+      <c r="D43" s="29" t="n"/>
+      <c r="E43" s="29" t="n"/>
+      <c r="F43" s="29" t="n"/>
+      <c r="G43" s="29" t="n"/>
+      <c r="H43" s="29" t="n"/>
+      <c r="I43" s="29" t="n"/>
     </row>
     <row r="44" ht="20" customHeight="1">
-      <c r="A44" s="24" t="n"/>
-      <c r="B44" s="24" t="n"/>
-      <c r="C44" s="24" t="n"/>
-      <c r="D44" s="24" t="n"/>
-      <c r="E44" s="24" t="n"/>
-      <c r="F44" s="24" t="n"/>
-      <c r="G44" s="24" t="n"/>
-      <c r="H44" s="24" t="n"/>
-      <c r="I44" s="24" t="n"/>
+      <c r="A44" s="29" t="n"/>
+      <c r="B44" s="29" t="n"/>
+      <c r="C44" s="29" t="n"/>
+      <c r="D44" s="29" t="n"/>
+      <c r="E44" s="29" t="n"/>
+      <c r="F44" s="29" t="n"/>
+      <c r="G44" s="29" t="n"/>
+      <c r="H44" s="29" t="n"/>
+      <c r="I44" s="29" t="n"/>
     </row>
     <row r="45" ht="20" customHeight="1">
-      <c r="A45" s="24" t="n"/>
-      <c r="B45" s="24" t="n"/>
-      <c r="C45" s="24" t="n"/>
-      <c r="D45" s="24" t="n"/>
-      <c r="E45" s="24" t="n"/>
-      <c r="F45" s="24" t="n"/>
-      <c r="G45" s="24" t="n"/>
-      <c r="H45" s="24" t="n"/>
-      <c r="I45" s="24" t="n"/>
+      <c r="A45" s="29" t="n"/>
+      <c r="B45" s="29" t="n"/>
+      <c r="C45" s="29" t="n"/>
+      <c r="D45" s="29" t="n"/>
+      <c r="E45" s="29" t="n"/>
+      <c r="F45" s="29" t="n"/>
+      <c r="G45" s="29" t="n"/>
+      <c r="H45" s="29" t="n"/>
+      <c r="I45" s="29" t="n"/>
     </row>
     <row r="46" ht="20" customHeight="1">
-      <c r="A46" s="24" t="n"/>
-      <c r="B46" s="24" t="n"/>
-      <c r="C46" s="24" t="n"/>
-      <c r="D46" s="24" t="n"/>
-      <c r="E46" s="24" t="n"/>
-      <c r="F46" s="24" t="n"/>
-      <c r="G46" s="24" t="n"/>
-      <c r="H46" s="24" t="n"/>
-      <c r="I46" s="24" t="n"/>
+      <c r="A46" s="29" t="n"/>
+      <c r="B46" s="29" t="n"/>
+      <c r="C46" s="29" t="n"/>
+      <c r="D46" s="29" t="n"/>
+      <c r="E46" s="29" t="n"/>
+      <c r="F46" s="29" t="n"/>
+      <c r="G46" s="29" t="n"/>
+      <c r="H46" s="29" t="n"/>
+      <c r="I46" s="29" t="n"/>
     </row>
     <row r="47" ht="20" customHeight="1">
-      <c r="A47" s="24" t="n"/>
-      <c r="B47" s="24" t="n"/>
-      <c r="C47" s="24" t="n"/>
-      <c r="D47" s="24" t="n"/>
-      <c r="E47" s="24" t="n"/>
-      <c r="F47" s="24" t="n"/>
-      <c r="G47" s="24" t="n"/>
-      <c r="H47" s="24" t="n"/>
-      <c r="I47" s="24" t="n"/>
+      <c r="A47" s="29" t="n"/>
+      <c r="B47" s="29" t="n"/>
+      <c r="C47" s="29" t="n"/>
+      <c r="D47" s="29" t="n"/>
+      <c r="E47" s="29" t="n"/>
+      <c r="F47" s="29" t="n"/>
+      <c r="G47" s="29" t="n"/>
+      <c r="H47" s="29" t="n"/>
+      <c r="I47" s="29" t="n"/>
     </row>
     <row r="48" ht="20" customHeight="1">
-      <c r="A48" s="24" t="n"/>
-      <c r="B48" s="24" t="n"/>
-      <c r="C48" s="24" t="n"/>
-      <c r="D48" s="24" t="n"/>
-      <c r="E48" s="24" t="n"/>
-      <c r="F48" s="24" t="n"/>
-      <c r="G48" s="24" t="n"/>
-      <c r="H48" s="24" t="n"/>
-      <c r="I48" s="24" t="n"/>
+      <c r="A48" s="29" t="n"/>
+      <c r="B48" s="29" t="n"/>
+      <c r="C48" s="29" t="n"/>
+      <c r="D48" s="29" t="n"/>
+      <c r="E48" s="29" t="n"/>
+      <c r="F48" s="29" t="n"/>
+      <c r="G48" s="29" t="n"/>
+      <c r="H48" s="29" t="n"/>
+      <c r="I48" s="29" t="n"/>
     </row>
     <row r="49" ht="20" customHeight="1">
-      <c r="A49" s="24" t="n"/>
-      <c r="B49" s="24" t="n"/>
-      <c r="C49" s="24" t="n"/>
-      <c r="D49" s="24" t="n"/>
-      <c r="E49" s="24" t="n"/>
-      <c r="F49" s="24" t="n"/>
-      <c r="G49" s="24" t="n"/>
-      <c r="H49" s="24" t="n"/>
-      <c r="I49" s="24" t="n"/>
+      <c r="A49" s="29" t="n"/>
+      <c r="B49" s="29" t="n"/>
+      <c r="C49" s="29" t="n"/>
+      <c r="D49" s="29" t="n"/>
+      <c r="E49" s="29" t="n"/>
+      <c r="F49" s="29" t="n"/>
+      <c r="G49" s="29" t="n"/>
+      <c r="H49" s="29" t="n"/>
+      <c r="I49" s="29" t="n"/>
     </row>
     <row r="50" ht="20" customHeight="1">
-      <c r="A50" s="24" t="n"/>
-      <c r="B50" s="24" t="n"/>
-      <c r="C50" s="24" t="n"/>
-      <c r="D50" s="24" t="n"/>
-      <c r="E50" s="24" t="n"/>
-      <c r="F50" s="24" t="n"/>
-      <c r="G50" s="24" t="n"/>
-      <c r="H50" s="24" t="n"/>
-      <c r="I50" s="24" t="n"/>
+      <c r="A50" s="29" t="n"/>
+      <c r="B50" s="29" t="n"/>
+      <c r="C50" s="29" t="n"/>
+      <c r="D50" s="29" t="n"/>
+      <c r="E50" s="29" t="n"/>
+      <c r="F50" s="29" t="n"/>
+      <c r="G50" s="29" t="n"/>
+      <c r="H50" s="29" t="n"/>
+      <c r="I50" s="29" t="n"/>
     </row>
     <row r="51" ht="20" customHeight="1">
-      <c r="A51" s="24" t="n"/>
-      <c r="B51" s="24" t="n"/>
-      <c r="C51" s="24" t="n"/>
-      <c r="D51" s="24" t="n"/>
-      <c r="E51" s="24" t="n"/>
-      <c r="F51" s="24" t="n"/>
-      <c r="G51" s="24" t="n"/>
-      <c r="H51" s="24" t="n"/>
-      <c r="I51" s="24" t="n"/>
+      <c r="A51" s="29" t="n"/>
+      <c r="B51" s="29" t="n"/>
+      <c r="C51" s="29" t="n"/>
+      <c r="D51" s="29" t="n"/>
+      <c r="E51" s="29" t="n"/>
+      <c r="F51" s="29" t="n"/>
+      <c r="G51" s="29" t="n"/>
+      <c r="H51" s="29" t="n"/>
+      <c r="I51" s="29" t="n"/>
     </row>
     <row r="52" ht="20" customHeight="1">
-      <c r="A52" s="24" t="n"/>
-      <c r="B52" s="24" t="n"/>
-      <c r="C52" s="24" t="n"/>
-      <c r="D52" s="24" t="n"/>
-      <c r="E52" s="24" t="n"/>
-      <c r="F52" s="24" t="n"/>
-      <c r="G52" s="24" t="n"/>
-      <c r="H52" s="24" t="n"/>
-      <c r="I52" s="24" t="n"/>
+      <c r="A52" s="29" t="n"/>
+      <c r="B52" s="29" t="n"/>
+      <c r="C52" s="29" t="n"/>
+      <c r="D52" s="29" t="n"/>
+      <c r="E52" s="29" t="n"/>
+      <c r="F52" s="29" t="n"/>
+      <c r="G52" s="29" t="n"/>
+      <c r="H52" s="29" t="n"/>
+      <c r="I52" s="29" t="n"/>
     </row>
     <row r="53" ht="20" customHeight="1">
-      <c r="A53" s="24" t="n"/>
-      <c r="B53" s="24" t="n"/>
-      <c r="C53" s="24" t="n"/>
-      <c r="D53" s="24" t="n"/>
-      <c r="E53" s="24" t="n"/>
-      <c r="F53" s="24" t="n"/>
-      <c r="G53" s="24" t="n"/>
-      <c r="H53" s="24" t="n"/>
-      <c r="I53" s="24" t="n"/>
+      <c r="A53" s="29" t="n"/>
+      <c r="B53" s="29" t="n"/>
+      <c r="C53" s="29" t="n"/>
+      <c r="D53" s="29" t="n"/>
+      <c r="E53" s="29" t="n"/>
+      <c r="F53" s="29" t="n"/>
+      <c r="G53" s="29" t="n"/>
+      <c r="H53" s="29" t="n"/>
+      <c r="I53" s="29" t="n"/>
     </row>
     <row r="54" ht="20" customHeight="1">
-      <c r="A54" s="24" t="n"/>
-      <c r="B54" s="24" t="n"/>
-      <c r="C54" s="24" t="n"/>
-      <c r="D54" s="24" t="n"/>
-      <c r="E54" s="24" t="n"/>
-      <c r="F54" s="24" t="n"/>
-      <c r="G54" s="24" t="n"/>
-      <c r="H54" s="24" t="n"/>
-      <c r="I54" s="24" t="n"/>
+      <c r="A54" s="29" t="n"/>
+      <c r="B54" s="29" t="n"/>
+      <c r="C54" s="29" t="n"/>
+      <c r="D54" s="29" t="n"/>
+      <c r="E54" s="29" t="n"/>
+      <c r="F54" s="29" t="n"/>
+      <c r="G54" s="29" t="n"/>
+      <c r="H54" s="29" t="n"/>
+      <c r="I54" s="29" t="n"/>
     </row>
     <row r="55" ht="20" customHeight="1">
-      <c r="A55" s="24" t="n"/>
-      <c r="B55" s="24" t="n"/>
-      <c r="C55" s="24" t="n"/>
-      <c r="D55" s="24" t="n"/>
-      <c r="E55" s="24" t="n"/>
-      <c r="F55" s="24" t="n"/>
-      <c r="G55" s="24" t="n"/>
-      <c r="H55" s="24" t="n"/>
-      <c r="I55" s="24" t="n"/>
+      <c r="A55" s="29" t="n"/>
+      <c r="B55" s="29" t="n"/>
+      <c r="C55" s="29" t="n"/>
+      <c r="D55" s="29" t="n"/>
+      <c r="E55" s="29" t="n"/>
+      <c r="F55" s="29" t="n"/>
+      <c r="G55" s="29" t="n"/>
+      <c r="H55" s="29" t="n"/>
+      <c r="I55" s="29" t="n"/>
     </row>
     <row r="56" ht="20" customHeight="1">
-      <c r="A56" s="24" t="n"/>
-      <c r="B56" s="24" t="n"/>
-      <c r="C56" s="24" t="n"/>
-      <c r="D56" s="24" t="n"/>
-      <c r="E56" s="24" t="n"/>
-      <c r="F56" s="24" t="n"/>
-      <c r="G56" s="24" t="n"/>
-      <c r="H56" s="24" t="n"/>
-      <c r="I56" s="24" t="n"/>
+      <c r="A56" s="29" t="n"/>
+      <c r="B56" s="29" t="n"/>
+      <c r="C56" s="29" t="n"/>
+      <c r="D56" s="29" t="n"/>
+      <c r="E56" s="29" t="n"/>
+      <c r="F56" s="29" t="n"/>
+      <c r="G56" s="29" t="n"/>
+      <c r="H56" s="29" t="n"/>
+      <c r="I56" s="29" t="n"/>
     </row>
     <row r="57" ht="20" customHeight="1">
-      <c r="A57" s="24" t="n"/>
-      <c r="B57" s="24" t="n"/>
-      <c r="C57" s="24" t="n"/>
-      <c r="D57" s="24" t="n"/>
-      <c r="E57" s="24" t="n"/>
-      <c r="F57" s="24" t="n"/>
-      <c r="G57" s="24" t="n"/>
-      <c r="H57" s="24" t="n"/>
-      <c r="I57" s="24" t="n"/>
+      <c r="A57" s="29" t="n"/>
+      <c r="B57" s="29" t="n"/>
+      <c r="C57" s="29" t="n"/>
+      <c r="D57" s="29" t="n"/>
+      <c r="E57" s="29" t="n"/>
+      <c r="F57" s="29" t="n"/>
+      <c r="G57" s="29" t="n"/>
+      <c r="H57" s="29" t="n"/>
+      <c r="I57" s="29" t="n"/>
     </row>
     <row r="58" ht="20" customHeight="1">
-      <c r="A58" s="24" t="n"/>
-      <c r="B58" s="24" t="n"/>
-      <c r="C58" s="24" t="n"/>
-      <c r="D58" s="24" t="n"/>
-      <c r="E58" s="24" t="n"/>
-      <c r="F58" s="24" t="n"/>
-      <c r="G58" s="24" t="n"/>
-      <c r="H58" s="24" t="n"/>
-      <c r="I58" s="24" t="n"/>
+      <c r="A58" s="29" t="n"/>
+      <c r="B58" s="29" t="n"/>
+      <c r="C58" s="29" t="n"/>
+      <c r="D58" s="29" t="n"/>
+      <c r="E58" s="29" t="n"/>
+      <c r="F58" s="29" t="n"/>
+      <c r="G58" s="29" t="n"/>
+      <c r="H58" s="29" t="n"/>
+      <c r="I58" s="29" t="n"/>
     </row>
     <row r="59" ht="20" customHeight="1">
-      <c r="A59" s="24" t="n"/>
-      <c r="B59" s="24" t="n"/>
-      <c r="C59" s="24" t="n"/>
-      <c r="D59" s="24" t="n"/>
-      <c r="E59" s="24" t="n"/>
-      <c r="F59" s="24" t="n"/>
-      <c r="G59" s="24" t="n"/>
-      <c r="H59" s="24" t="n"/>
-      <c r="I59" s="24" t="n"/>
+      <c r="A59" s="29" t="n"/>
+      <c r="B59" s="29" t="n"/>
+      <c r="C59" s="29" t="n"/>
+      <c r="D59" s="29" t="n"/>
+      <c r="E59" s="29" t="n"/>
+      <c r="F59" s="29" t="n"/>
+      <c r="G59" s="29" t="n"/>
+      <c r="H59" s="29" t="n"/>
+      <c r="I59" s="29" t="n"/>
     </row>
     <row r="60" ht="20" customHeight="1">
-      <c r="A60" s="24" t="n"/>
-      <c r="B60" s="24" t="n"/>
-      <c r="C60" s="24" t="n"/>
-      <c r="D60" s="24" t="n"/>
-      <c r="E60" s="24" t="n"/>
-      <c r="F60" s="24" t="n"/>
-      <c r="G60" s="24" t="n"/>
-      <c r="H60" s="24" t="n"/>
-      <c r="I60" s="24" t="n"/>
+      <c r="A60" s="29" t="n"/>
+      <c r="B60" s="29" t="n"/>
+      <c r="C60" s="29" t="n"/>
+      <c r="D60" s="29" t="n"/>
+      <c r="E60" s="29" t="n"/>
+      <c r="F60" s="29" t="n"/>
+      <c r="G60" s="29" t="n"/>
+      <c r="H60" s="29" t="n"/>
+      <c r="I60" s="29" t="n"/>
     </row>
     <row r="61" ht="20" customHeight="1">
-      <c r="A61" s="24" t="n"/>
-      <c r="B61" s="24" t="n"/>
-      <c r="C61" s="24" t="n"/>
-      <c r="D61" s="24" t="n"/>
-      <c r="E61" s="24" t="n"/>
-      <c r="F61" s="24" t="n"/>
-      <c r="G61" s="24" t="n"/>
-      <c r="H61" s="24" t="n"/>
-      <c r="I61" s="24" t="n"/>
+      <c r="A61" s="29" t="n"/>
+      <c r="B61" s="29" t="n"/>
+      <c r="C61" s="29" t="n"/>
+      <c r="D61" s="29" t="n"/>
+      <c r="E61" s="29" t="n"/>
+      <c r="F61" s="29" t="n"/>
+      <c r="G61" s="29" t="n"/>
+      <c r="H61" s="29" t="n"/>
+      <c r="I61" s="29" t="n"/>
     </row>
     <row r="62" ht="20" customHeight="1">
-      <c r="A62" s="24" t="n"/>
-      <c r="B62" s="24" t="n"/>
-      <c r="C62" s="24" t="n"/>
-      <c r="D62" s="24" t="n"/>
-      <c r="E62" s="24" t="n"/>
-      <c r="F62" s="24" t="n"/>
-      <c r="G62" s="24" t="n"/>
-      <c r="H62" s="24" t="n"/>
-      <c r="I62" s="24" t="n"/>
+      <c r="A62" s="29" t="n"/>
+      <c r="B62" s="29" t="n"/>
+      <c r="C62" s="29" t="n"/>
+      <c r="D62" s="29" t="n"/>
+      <c r="E62" s="29" t="n"/>
+      <c r="F62" s="29" t="n"/>
+      <c r="G62" s="29" t="n"/>
+      <c r="H62" s="29" t="n"/>
+      <c r="I62" s="29" t="n"/>
     </row>
     <row r="63" ht="20" customHeight="1">
-      <c r="A63" s="24" t="n"/>
-      <c r="B63" s="24" t="n"/>
-      <c r="C63" s="24" t="n"/>
-      <c r="D63" s="24" t="n"/>
-      <c r="E63" s="24" t="n"/>
-      <c r="F63" s="24" t="n"/>
-      <c r="G63" s="24" t="n"/>
-      <c r="H63" s="24" t="n"/>
-      <c r="I63" s="24" t="n"/>
+      <c r="A63" s="29" t="n"/>
+      <c r="B63" s="29" t="n"/>
+      <c r="C63" s="29" t="n"/>
+      <c r="D63" s="29" t="n"/>
+      <c r="E63" s="29" t="n"/>
+      <c r="F63" s="29" t="n"/>
+      <c r="G63" s="29" t="n"/>
+      <c r="H63" s="29" t="n"/>
+      <c r="I63" s="29" t="n"/>
     </row>
     <row r="64" ht="20" customHeight="1">
-      <c r="A64" s="24" t="n"/>
-      <c r="B64" s="24" t="n"/>
-      <c r="C64" s="24" t="n"/>
-      <c r="D64" s="24" t="n"/>
-      <c r="E64" s="24" t="n"/>
-      <c r="F64" s="24" t="n"/>
-      <c r="G64" s="24" t="n"/>
-      <c r="H64" s="24" t="n"/>
-      <c r="I64" s="24" t="n"/>
+      <c r="A64" s="29" t="n"/>
+      <c r="B64" s="29" t="n"/>
+      <c r="C64" s="29" t="n"/>
+      <c r="D64" s="29" t="n"/>
+      <c r="E64" s="29" t="n"/>
+      <c r="F64" s="29" t="n"/>
+      <c r="G64" s="29" t="n"/>
+      <c r="H64" s="29" t="n"/>
+      <c r="I64" s="29" t="n"/>
     </row>
     <row r="65" ht="20" customHeight="1">
-      <c r="A65" s="24" t="n"/>
-      <c r="B65" s="24" t="n"/>
-      <c r="C65" s="24" t="n"/>
-      <c r="D65" s="24" t="n"/>
-      <c r="E65" s="24" t="n"/>
-      <c r="F65" s="24" t="n"/>
-      <c r="G65" s="24" t="n"/>
-      <c r="H65" s="24" t="n"/>
-      <c r="I65" s="24" t="n"/>
+      <c r="A65" s="29" t="n"/>
+      <c r="B65" s="29" t="n"/>
+      <c r="C65" s="29" t="n"/>
+      <c r="D65" s="29" t="n"/>
+      <c r="E65" s="29" t="n"/>
+      <c r="F65" s="29" t="n"/>
+      <c r="G65" s="29" t="n"/>
+      <c r="H65" s="29" t="n"/>
+      <c r="I65" s="29" t="n"/>
     </row>
     <row r="66" ht="20" customHeight="1">
-      <c r="A66" s="24" t="n"/>
-      <c r="B66" s="24" t="n"/>
-      <c r="C66" s="24" t="n"/>
-      <c r="D66" s="24" t="n"/>
-      <c r="E66" s="24" t="n"/>
-      <c r="F66" s="24" t="n"/>
-      <c r="G66" s="24" t="n"/>
-      <c r="H66" s="24" t="n"/>
-      <c r="I66" s="24" t="n"/>
+      <c r="A66" s="29" t="n"/>
+      <c r="B66" s="29" t="n"/>
+      <c r="C66" s="29" t="n"/>
+      <c r="D66" s="29" t="n"/>
+      <c r="E66" s="29" t="n"/>
+      <c r="F66" s="29" t="n"/>
+      <c r="G66" s="29" t="n"/>
+      <c r="H66" s="29" t="n"/>
+      <c r="I66" s="29" t="n"/>
     </row>
     <row r="67" ht="20" customHeight="1">
-      <c r="A67" s="24" t="n"/>
-      <c r="B67" s="24" t="n"/>
-      <c r="C67" s="24" t="n"/>
-      <c r="D67" s="24" t="n"/>
-      <c r="E67" s="24" t="n"/>
-      <c r="F67" s="24" t="n"/>
-      <c r="G67" s="24" t="n"/>
-      <c r="H67" s="24" t="n"/>
-      <c r="I67" s="24" t="n"/>
+      <c r="A67" s="29" t="n"/>
+      <c r="B67" s="29" t="n"/>
+      <c r="C67" s="29" t="n"/>
+      <c r="D67" s="29" t="n"/>
+      <c r="E67" s="29" t="n"/>
+      <c r="F67" s="29" t="n"/>
+      <c r="G67" s="29" t="n"/>
+      <c r="H67" s="29" t="n"/>
+      <c r="I67" s="29" t="n"/>
     </row>
     <row r="68" ht="20" customHeight="1">
-      <c r="A68" s="24" t="n"/>
-      <c r="B68" s="24" t="n"/>
-      <c r="C68" s="24" t="n"/>
-      <c r="D68" s="24" t="n"/>
-      <c r="E68" s="24" t="n"/>
-      <c r="F68" s="24" t="n"/>
-      <c r="G68" s="24" t="n"/>
-      <c r="H68" s="24" t="n"/>
-      <c r="I68" s="24" t="n"/>
+      <c r="A68" s="29" t="n"/>
+      <c r="B68" s="29" t="n"/>
+      <c r="C68" s="29" t="n"/>
+      <c r="D68" s="29" t="n"/>
+      <c r="E68" s="29" t="n"/>
+      <c r="F68" s="29" t="n"/>
+      <c r="G68" s="29" t="n"/>
+      <c r="H68" s="29" t="n"/>
+      <c r="I68" s="29" t="n"/>
     </row>
     <row r="69" ht="20" customHeight="1">
-      <c r="A69" s="24" t="n"/>
-      <c r="B69" s="24" t="n"/>
-      <c r="C69" s="24" t="n"/>
-      <c r="D69" s="24" t="n"/>
-      <c r="E69" s="24" t="n"/>
-      <c r="F69" s="24" t="n"/>
-      <c r="G69" s="24" t="n"/>
-      <c r="H69" s="24" t="n"/>
-      <c r="I69" s="24" t="n"/>
+      <c r="A69" s="29" t="n"/>
+      <c r="B69" s="29" t="n"/>
+      <c r="C69" s="29" t="n"/>
+      <c r="D69" s="29" t="n"/>
+      <c r="E69" s="29" t="n"/>
+      <c r="F69" s="29" t="n"/>
+      <c r="G69" s="29" t="n"/>
+      <c r="H69" s="29" t="n"/>
+      <c r="I69" s="29" t="n"/>
     </row>
     <row r="70" ht="20" customHeight="1">
-      <c r="A70" s="24" t="n"/>
-      <c r="B70" s="24" t="n"/>
-      <c r="C70" s="24" t="n"/>
-      <c r="D70" s="24" t="n"/>
-      <c r="E70" s="24" t="n"/>
-      <c r="F70" s="24" t="n"/>
-      <c r="G70" s="24" t="n"/>
-      <c r="H70" s="24" t="n"/>
-      <c r="I70" s="24" t="n"/>
+      <c r="A70" s="29" t="n"/>
+      <c r="B70" s="29" t="n"/>
+      <c r="C70" s="29" t="n"/>
+      <c r="D70" s="29" t="n"/>
+      <c r="E70" s="29" t="n"/>
+      <c r="F70" s="29" t="n"/>
+      <c r="G70" s="29" t="n"/>
+      <c r="H70" s="29" t="n"/>
+      <c r="I70" s="29" t="n"/>
     </row>
     <row r="71" ht="20" customHeight="1">
-      <c r="A71" s="24" t="n"/>
-      <c r="B71" s="24" t="n"/>
-      <c r="C71" s="24" t="n"/>
-      <c r="D71" s="24" t="n"/>
-      <c r="E71" s="24" t="n"/>
-      <c r="F71" s="24" t="n"/>
-      <c r="G71" s="24" t="n"/>
-      <c r="H71" s="24" t="n"/>
-      <c r="I71" s="24" t="n"/>
+      <c r="A71" s="29" t="n"/>
+      <c r="B71" s="29" t="n"/>
+      <c r="C71" s="29" t="n"/>
+      <c r="D71" s="29" t="n"/>
+      <c r="E71" s="29" t="n"/>
+      <c r="F71" s="29" t="n"/>
+      <c r="G71" s="29" t="n"/>
+      <c r="H71" s="29" t="n"/>
+      <c r="I71" s="29" t="n"/>
+    </row>
+    <row r="72" ht="20" customHeight="1">
+      <c r="A72" s="29" t="n"/>
+      <c r="B72" s="29" t="n"/>
+      <c r="C72" s="29" t="n"/>
+      <c r="D72" s="29" t="n"/>
+      <c r="E72" s="29" t="n"/>
+      <c r="F72" s="29" t="n"/>
+      <c r="G72" s="29" t="n"/>
+      <c r="H72" s="29" t="n"/>
+      <c r="I72" s="29" t="n"/>
+    </row>
+    <row r="73" ht="20" customHeight="1">
+      <c r="A73" s="29" t="n"/>
+      <c r="B73" s="29" t="n"/>
+      <c r="C73" s="29" t="n"/>
+      <c r="D73" s="29" t="n"/>
+      <c r="E73" s="29" t="n"/>
+      <c r="F73" s="29" t="n"/>
+      <c r="G73" s="29" t="n"/>
+      <c r="H73" s="29" t="n"/>
+      <c r="I73" s="29" t="n"/>
+    </row>
+    <row r="74" ht="20" customHeight="1">
+      <c r="A74" s="29" t="n"/>
+      <c r="B74" s="29" t="n"/>
+      <c r="C74" s="29" t="n"/>
+      <c r="D74" s="29" t="n"/>
+      <c r="E74" s="29" t="n"/>
+      <c r="F74" s="29" t="n"/>
+      <c r="G74" s="29" t="n"/>
+      <c r="H74" s="29" t="n"/>
+      <c r="I74" s="29" t="n"/>
+    </row>
+    <row r="75" ht="20" customHeight="1">
+      <c r="A75" s="29" t="n"/>
+      <c r="B75" s="29" t="n"/>
+      <c r="C75" s="29" t="n"/>
+      <c r="D75" s="29" t="n"/>
+      <c r="E75" s="29" t="n"/>
+      <c r="F75" s="29" t="n"/>
+      <c r="G75" s="29" t="n"/>
+      <c r="H75" s="29" t="n"/>
+      <c r="I75" s="29" t="n"/>
+    </row>
+    <row r="76" ht="20" customHeight="1">
+      <c r="A76" s="29" t="n"/>
+      <c r="B76" s="29" t="n"/>
+      <c r="C76" s="29" t="n"/>
+      <c r="D76" s="29" t="n"/>
+      <c r="E76" s="29" t="n"/>
+      <c r="F76" s="29" t="n"/>
+      <c r="G76" s="29" t="n"/>
+      <c r="H76" s="29" t="n"/>
+      <c r="I76" s="29" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A10:I71"/>
-  <mergeCells count="22">
+  <autoFilter ref="A15:I76"/>
+  <mergeCells count="26">
     <mergeCell ref="I5"/>
     <mergeCell ref="C6:D6"/>
     <mergeCell ref="I4"/>
     <mergeCell ref="C5:D5"/>
     <mergeCell ref="E5:F5"/>
+    <mergeCell ref="A12:C12"/>
     <mergeCell ref="A6:B6"/>
     <mergeCell ref="C4:D4"/>
     <mergeCell ref="E4:F4"/>
@@ -1887,17 +2006,20 @@
     <mergeCell ref="G7:H7"/>
     <mergeCell ref="I6"/>
     <mergeCell ref="G6:H6"/>
+    <mergeCell ref="A10:C10"/>
     <mergeCell ref="E6:F6"/>
     <mergeCell ref="A5:B5"/>
     <mergeCell ref="G5:H5"/>
+    <mergeCell ref="A9:C9"/>
     <mergeCell ref="I7"/>
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="G4:H4"/>
+    <mergeCell ref="A11:C11"/>
     <mergeCell ref="C7:D7"/>
     <mergeCell ref="E7:F7"/>
     <mergeCell ref="A1:I1"/>
   </mergeCells>
-  <conditionalFormatting sqref="D11:D71">
+  <conditionalFormatting sqref="A10:C10">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Critical"</formula>
     </cfRule>
@@ -1911,37 +2033,51 @@
       <formula>"Low"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E11:E71">
+  <conditionalFormatting sqref="D16:D76">
     <cfRule type="cellIs" priority="5" operator="equal" dxfId="4">
+      <formula>"Critical"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="6" operator="equal" dxfId="5">
+      <formula>"High"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="7" operator="equal" dxfId="6">
+      <formula>"Medium"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="8" operator="equal" dxfId="7">
+      <formula>"Low"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E16:E76">
+    <cfRule type="cellIs" priority="9" operator="equal" dxfId="8">
       <formula>"New"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="6" operator="equal" dxfId="5">
+    <cfRule type="cellIs" priority="10" operator="equal" dxfId="9">
       <formula>"In Review"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="7" operator="equal" dxfId="6">
+    <cfRule type="cellIs" priority="11" operator="equal" dxfId="10">
       <formula>"Approved"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="8" operator="equal" dxfId="7">
+    <cfRule type="cellIs" priority="12" operator="equal" dxfId="11">
       <formula>"Scheduled"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="9" operator="equal" dxfId="8">
+    <cfRule type="cellIs" priority="13" operator="equal" dxfId="12">
       <formula>"In Progress"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="10" operator="equal" dxfId="9">
+    <cfRule type="cellIs" priority="14" operator="equal" dxfId="13">
       <formula>"Completed"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="11" operator="equal" dxfId="10">
+    <cfRule type="cellIs" priority="15" operator="equal" dxfId="14">
       <formula>"Blocked"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="12" operator="equal" dxfId="11">
+    <cfRule type="cellIs" priority="16" operator="equal" dxfId="15">
       <formula>"Rejected"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="D11:D71" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="D16:D76" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Critical,High,Medium,Low"</formula1>
     </dataValidation>
-    <dataValidation sqref="E11:E71" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E16:E76" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"New,In Review,Approved,Scheduled,In Progress,Completed,Blocked,Rejected"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>